<commit_message>
Add ML dashboard final work
</commit_message>
<xml_diff>
--- a/Camps_Detailles.xlsx
+++ b/Camps_Detailles.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9303"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Desktop\Scouts\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{189A2AB6-D21A-4E56-A791-91C7C278396F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
   <si>
     <t>Saison</t>
   </si>
@@ -62,12 +56,36 @@
   </si>
   <si>
     <t>Camp préparatoire</t>
+  </si>
+  <si>
+    <t>camp_code</t>
+  </si>
+  <si>
+    <t>Camp_printemps_2023-2024</t>
+  </si>
+  <si>
+    <t>Camp_été_2023-2024</t>
+  </si>
+  <si>
+    <t>Camp_printemps_2024-2025</t>
+  </si>
+  <si>
+    <t>Camp_été_jeunes_2024-2025</t>
+  </si>
+  <si>
+    <t>Camp_été_avancé_2024-2025</t>
+  </si>
+  <si>
+    <t>Camp_mobile_2024-2025</t>
+  </si>
+  <si>
+    <t>Camp_préparatoire_2025-2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -414,25 +432,26 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.109375" customWidth="1"/>
     <col min="2" max="2" width="27.21875" customWidth="1"/>
     <col min="3" max="3" width="32" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
     <col min="5" max="5" width="38.88671875" customWidth="1"/>
+    <col min="6" max="6" width="27.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -448,8 +467,11 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="F1" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>5</v>
       </c>
@@ -465,8 +487,11 @@
       <c r="E2" s="1">
         <v>8200</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="F2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>5</v>
       </c>
@@ -482,8 +507,11 @@
       <c r="E3" s="1">
         <v>18000</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="F3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>8</v>
       </c>
@@ -499,8 +527,11 @@
       <c r="E4" s="1">
         <v>10500</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="F4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>8</v>
       </c>
@@ -516,8 +547,11 @@
       <c r="E5" s="1">
         <v>11500</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="66" x14ac:dyDescent="0.3">
+      <c r="F5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
@@ -533,8 +567,11 @@
       <c r="E6" s="1">
         <v>13500</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="F6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>8</v>
       </c>
@@ -550,8 +587,11 @@
       <c r="E7" s="1">
         <v>2000</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="F7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>12</v>
       </c>
@@ -566,6 +606,9 @@
       </c>
       <c r="E8" s="1">
         <v>2000</v>
+      </c>
+      <c r="F8" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>